<commit_message>
updated graph travelsal, moved embedding class to embedding.py file
</commit_message>
<xml_diff>
--- a/docs/Project_Workload.xlsx
+++ b/docs/Project_Workload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gagan/Projects/info_698/info-698-hybrid-rag/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDEE05D-7FEC-B541-B170-23B5E9A05022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{141DC179-CEE3-4D42-8FF4-F8AFBCE5C6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="24240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1204,12 +1204,30 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="13" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1224,24 +1242,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1809,29 +1809,29 @@
       <c r="E1" s="9"/>
       <c r="F1" s="10"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="118" t="s">
+      <c r="I1" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
       <c r="P1" s="13"/>
-      <c r="Q1" s="117">
+      <c r="Q1" s="115">
         <f>DATE(2025,9,15)</f>
         <v>45915</v>
       </c>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
+      <c r="R1" s="115"/>
+      <c r="S1" s="115"/>
+      <c r="T1" s="115"/>
+      <c r="U1" s="115"/>
+      <c r="V1" s="115"/>
+      <c r="W1" s="115"/>
+      <c r="X1" s="115"/>
+      <c r="Y1" s="115"/>
+      <c r="Z1" s="115"/>
       <c r="AJ1" t="s">
         <v>2</v>
       </c>
@@ -1846,28 +1846,28 @@
       <c r="D2" s="11"/>
       <c r="E2" s="12"/>
       <c r="F2" s="11"/>
-      <c r="I2" s="118" t="s">
+      <c r="I2" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="118"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118"/>
-      <c r="O2" s="118"/>
+      <c r="J2" s="116"/>
+      <c r="K2" s="116"/>
+      <c r="L2" s="116"/>
+      <c r="M2" s="116"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="116"/>
       <c r="P2" s="13"/>
-      <c r="Q2" s="116">
+      <c r="Q2" s="114">
         <v>4</v>
       </c>
-      <c r="R2" s="116"/>
-      <c r="S2" s="116"/>
-      <c r="T2" s="116"/>
-      <c r="U2" s="116"/>
-      <c r="V2" s="116"/>
-      <c r="W2" s="116"/>
-      <c r="X2" s="116"/>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
+      <c r="R2" s="114"/>
+      <c r="S2" s="114"/>
+      <c r="T2" s="114"/>
+      <c r="U2" s="114"/>
+      <c r="V2" s="114"/>
+      <c r="W2" s="114"/>
+      <c r="X2" s="114"/>
+      <c r="Y2" s="114"/>
+      <c r="Z2" s="114"/>
     </row>
     <row r="3" spans="1:64" s="15" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4"/>
@@ -1879,102 +1879,102 @@
       <c r="A4" s="5"/>
       <c r="B4" s="18"/>
       <c r="E4" s="19"/>
-      <c r="I4" s="120">
+      <c r="I4" s="110">
         <f>I5</f>
         <v>45936</v>
       </c>
-      <c r="J4" s="120"/>
-      <c r="K4" s="120"/>
-      <c r="L4" s="120"/>
-      <c r="M4" s="120"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="121"/>
-      <c r="P4" s="119">
+      <c r="J4" s="110"/>
+      <c r="K4" s="110"/>
+      <c r="L4" s="110"/>
+      <c r="M4" s="110"/>
+      <c r="N4" s="110"/>
+      <c r="O4" s="111"/>
+      <c r="P4" s="109">
         <f>P5</f>
         <v>45943</v>
       </c>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="120"/>
-      <c r="S4" s="120"/>
-      <c r="T4" s="120"/>
-      <c r="U4" s="120"/>
-      <c r="V4" s="121"/>
-      <c r="W4" s="119">
+      <c r="Q4" s="110"/>
+      <c r="R4" s="110"/>
+      <c r="S4" s="110"/>
+      <c r="T4" s="110"/>
+      <c r="U4" s="110"/>
+      <c r="V4" s="111"/>
+      <c r="W4" s="109">
         <f>W5</f>
         <v>45950</v>
       </c>
-      <c r="X4" s="120"/>
-      <c r="Y4" s="120"/>
-      <c r="Z4" s="120"/>
-      <c r="AA4" s="120"/>
-      <c r="AB4" s="120"/>
-      <c r="AC4" s="121"/>
-      <c r="AD4" s="119">
+      <c r="X4" s="110"/>
+      <c r="Y4" s="110"/>
+      <c r="Z4" s="110"/>
+      <c r="AA4" s="110"/>
+      <c r="AB4" s="110"/>
+      <c r="AC4" s="111"/>
+      <c r="AD4" s="109">
         <f>AD5</f>
         <v>45957</v>
       </c>
-      <c r="AE4" s="120"/>
-      <c r="AF4" s="120"/>
-      <c r="AG4" s="120"/>
-      <c r="AH4" s="120"/>
-      <c r="AI4" s="120"/>
-      <c r="AJ4" s="121"/>
-      <c r="AK4" s="119">
+      <c r="AE4" s="110"/>
+      <c r="AF4" s="110"/>
+      <c r="AG4" s="110"/>
+      <c r="AH4" s="110"/>
+      <c r="AI4" s="110"/>
+      <c r="AJ4" s="111"/>
+      <c r="AK4" s="109">
         <f>AK5</f>
         <v>45964</v>
       </c>
-      <c r="AL4" s="120"/>
-      <c r="AM4" s="120"/>
-      <c r="AN4" s="120"/>
-      <c r="AO4" s="120"/>
-      <c r="AP4" s="120"/>
-      <c r="AQ4" s="121"/>
-      <c r="AR4" s="119">
+      <c r="AL4" s="110"/>
+      <c r="AM4" s="110"/>
+      <c r="AN4" s="110"/>
+      <c r="AO4" s="110"/>
+      <c r="AP4" s="110"/>
+      <c r="AQ4" s="111"/>
+      <c r="AR4" s="109">
         <f>AR5</f>
         <v>45971</v>
       </c>
-      <c r="AS4" s="120"/>
-      <c r="AT4" s="120"/>
-      <c r="AU4" s="120"/>
-      <c r="AV4" s="120"/>
-      <c r="AW4" s="120"/>
-      <c r="AX4" s="121"/>
-      <c r="AY4" s="119">
+      <c r="AS4" s="110"/>
+      <c r="AT4" s="110"/>
+      <c r="AU4" s="110"/>
+      <c r="AV4" s="110"/>
+      <c r="AW4" s="110"/>
+      <c r="AX4" s="111"/>
+      <c r="AY4" s="109">
         <f>AY5</f>
         <v>45978</v>
       </c>
-      <c r="AZ4" s="120"/>
-      <c r="BA4" s="120"/>
-      <c r="BB4" s="120"/>
-      <c r="BC4" s="120"/>
-      <c r="BD4" s="120"/>
-      <c r="BE4" s="121"/>
-      <c r="BF4" s="119">
+      <c r="AZ4" s="110"/>
+      <c r="BA4" s="110"/>
+      <c r="BB4" s="110"/>
+      <c r="BC4" s="110"/>
+      <c r="BD4" s="110"/>
+      <c r="BE4" s="111"/>
+      <c r="BF4" s="109">
         <f>BF5</f>
         <v>45985</v>
       </c>
-      <c r="BG4" s="120"/>
-      <c r="BH4" s="120"/>
-      <c r="BI4" s="120"/>
-      <c r="BJ4" s="120"/>
-      <c r="BK4" s="120"/>
-      <c r="BL4" s="120"/>
+      <c r="BG4" s="110"/>
+      <c r="BH4" s="110"/>
+      <c r="BI4" s="110"/>
+      <c r="BJ4" s="110"/>
+      <c r="BK4" s="110"/>
+      <c r="BL4" s="110"/>
     </row>
     <row r="5" spans="1:64" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="115"/>
-      <c r="B5" s="113" t="s">
+      <c r="A5" s="121"/>
+      <c r="B5" s="119" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="111" t="s">
+      <c r="C5" s="117" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="109" t="s">
+      <c r="D5" s="112" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="109" t="s">
+      <c r="E5" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="109" t="s">
+      <c r="F5" s="112" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="20">
@@ -2203,12 +2203,12 @@
       </c>
     </row>
     <row r="6" spans="1:64" s="15" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="115"/>
-      <c r="B6" s="114"/>
-      <c r="C6" s="112"/>
-      <c r="D6" s="110"/>
-      <c r="E6" s="110"/>
-      <c r="F6" s="110"/>
+      <c r="A6" s="121"/>
+      <c r="B6" s="120"/>
+      <c r="C6" s="118"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="113"/>
       <c r="I6" s="23" t="str">
         <f t="shared" ref="I6:AN6" si="3">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>M</v>
@@ -3220,13 +3220,13 @@
         <v>45947</v>
       </c>
       <c r="F17" s="48">
-        <f>E17+13</f>
-        <v>45960</v>
+        <f>E17+14</f>
+        <v>45961</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="3">
         <f t="shared" si="5"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="34"/>
@@ -3301,13 +3301,13 @@
         <v>45947</v>
       </c>
       <c r="F18" s="48">
-        <f t="shared" ref="F18:F19" si="6">E18+13</f>
-        <v>45960</v>
+        <f t="shared" ref="F18:F19" si="6">E18+14</f>
+        <v>45961</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="3">
         <f t="shared" si="5"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="34"/>
@@ -3383,12 +3383,12 @@
       </c>
       <c r="F19" s="48">
         <f t="shared" si="6"/>
-        <v>45960</v>
+        <v>45961</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="3">
         <f t="shared" si="5"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="34"/>
@@ -3529,11 +3529,11 @@
       <c r="D21" s="56"/>
       <c r="E21" s="57">
         <f>F19</f>
-        <v>45960</v>
+        <v>45961</v>
       </c>
       <c r="F21" s="57">
         <f>E21+8</f>
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="3">
@@ -3608,11 +3608,11 @@
       <c r="D22" s="56"/>
       <c r="E22" s="57">
         <f>E21</f>
-        <v>45960</v>
+        <v>45961</v>
       </c>
       <c r="F22" s="57">
         <f>E22+8</f>
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="3">
@@ -3758,11 +3758,11 @@
       <c r="D24" s="65"/>
       <c r="E24" s="66">
         <f>F22</f>
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="F24" s="66">
         <f>E24+7</f>
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="3">
@@ -3837,11 +3837,11 @@
       <c r="D25" s="65"/>
       <c r="E25" s="66">
         <f>E24</f>
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="F25" s="66">
         <f t="shared" ref="F25:F26" si="7">E25+7</f>
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="3">
@@ -3916,11 +3916,11 @@
       <c r="D26" s="65"/>
       <c r="E26" s="66">
         <f>E25</f>
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="F26" s="66">
         <f t="shared" si="7"/>
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="3">
@@ -4066,11 +4066,11 @@
       <c r="D28" s="84"/>
       <c r="E28" s="85">
         <f>F26</f>
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="F28" s="85">
         <f>E28+7</f>
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="3">
@@ -4145,11 +4145,11 @@
       <c r="D29" s="84"/>
       <c r="E29" s="85">
         <f>E28</f>
-        <v>45975</v>
+        <v>45976</v>
       </c>
       <c r="F29" s="85">
         <f>E29+7</f>
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="3">
@@ -4295,11 +4295,11 @@
       <c r="D31" s="93"/>
       <c r="E31" s="94">
         <f>F29</f>
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="F31" s="94">
         <f>E31+7</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="3">
@@ -4374,11 +4374,11 @@
       <c r="D32" s="93"/>
       <c r="E32" s="94">
         <f>E31</f>
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="F32" s="94">
         <f>E32+7</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="3">
@@ -4524,11 +4524,11 @@
       <c r="D34" s="102"/>
       <c r="E34" s="103">
         <f>F32</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="F34" s="103">
         <f>E34+7</f>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="3">
@@ -4603,11 +4603,11 @@
       <c r="D35" s="102"/>
       <c r="E35" s="103">
         <f>E34</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="F35" s="103">
         <f t="shared" ref="F35:F37" si="8">E35+7</f>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="3">
@@ -4682,11 +4682,11 @@
       <c r="D36" s="102"/>
       <c r="E36" s="103">
         <f>E35</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="F36" s="103">
         <f t="shared" si="8"/>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="3">
@@ -4761,11 +4761,11 @@
       <c r="D37" s="102"/>
       <c r="E37" s="103">
         <f>E36</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="F37" s="103">
         <f t="shared" si="8"/>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="3">
@@ -4911,11 +4911,11 @@
       <c r="D39" s="65"/>
       <c r="E39" s="66">
         <f>E37</f>
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="F39" s="66">
         <f>F37</f>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="3">
@@ -5061,11 +5061,11 @@
       <c r="D41" s="93"/>
       <c r="E41" s="94">
         <f>F39</f>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="F41" s="94">
         <f>F39</f>
-        <v>45996</v>
+        <v>45997</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="3">
@@ -5131,6 +5131,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="Q2:Z2"/>
+    <mergeCell ref="Q1:Z1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="I2:O2"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
@@ -5139,16 +5149,6 @@
     <mergeCell ref="AK4:AQ4"/>
     <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="Q2:Z2"/>
-    <mergeCell ref="Q1:Z1"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="I2:O2"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A5:A6"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D41">
     <cfRule type="dataBar" priority="26">
@@ -5818,6 +5818,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006B8B2E08FBA2934085025AE2CC2D4FCF" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8d5915535425329bcbd771e38b5089a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d9b4d3a9-89d7-4752-9f66-1c4049782483" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a4a6479488fcfa1ea26509531871ed87" ns3:_="">
     <xsd:import namespace="d9b4d3a9-89d7-4752-9f66-1c4049782483"/>
@@ -5967,22 +5982,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E186200E-CA11-482F-967A-1FD62478FEA5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6000,23 +6017,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
Updated RREADME.md, added docker support, enabled tracing
</commit_message>
<xml_diff>
--- a/docs/Project_Workload.xlsx
+++ b/docs/Project_Workload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gagan/Projects/info_698/info-698-hybrid-rag/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1122B2B-864C-9D4C-BDC7-90FDC72EE838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7ABFBE3-BF97-AC43-892D-8B6F83F6A0E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="24240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="104">
   <si>
     <t>A Hybrid RAG System with Graph Based Context Retrieval</t>
   </si>
@@ -360,6 +360,9 @@
   </si>
   <si>
     <t>Explore evaluation strategies</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -1207,6 +1210,36 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="166" fontId="13" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1215,36 +1248,6 @@
     </xf>
     <xf numFmtId="166" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1814,29 +1817,29 @@
       <c r="E1" s="9"/>
       <c r="F1" s="10"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="116" t="s">
+      <c r="I1" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
       <c r="P1" s="13"/>
-      <c r="Q1" s="115">
+      <c r="Q1" s="117">
         <f>DATE(2025,9,15)</f>
         <v>45915</v>
       </c>
-      <c r="R1" s="115"/>
-      <c r="S1" s="115"/>
-      <c r="T1" s="115"/>
-      <c r="U1" s="115"/>
-      <c r="V1" s="115"/>
-      <c r="W1" s="115"/>
-      <c r="X1" s="115"/>
-      <c r="Y1" s="115"/>
-      <c r="Z1" s="115"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
       <c r="AJ1" t="s">
         <v>2</v>
       </c>
@@ -1851,28 +1854,28 @@
       <c r="D2" s="11"/>
       <c r="E2" s="12"/>
       <c r="F2" s="11"/>
-      <c r="I2" s="116" t="s">
+      <c r="I2" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="116"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
-      <c r="O2" s="116"/>
+      <c r="J2" s="118"/>
+      <c r="K2" s="118"/>
+      <c r="L2" s="118"/>
+      <c r="M2" s="118"/>
+      <c r="N2" s="118"/>
+      <c r="O2" s="118"/>
       <c r="P2" s="13"/>
-      <c r="Q2" s="114">
+      <c r="Q2" s="116">
         <v>4</v>
       </c>
-      <c r="R2" s="114"/>
-      <c r="S2" s="114"/>
-      <c r="T2" s="114"/>
-      <c r="U2" s="114"/>
-      <c r="V2" s="114"/>
-      <c r="W2" s="114"/>
-      <c r="X2" s="114"/>
-      <c r="Y2" s="114"/>
-      <c r="Z2" s="114"/>
+      <c r="R2" s="116"/>
+      <c r="S2" s="116"/>
+      <c r="T2" s="116"/>
+      <c r="U2" s="116"/>
+      <c r="V2" s="116"/>
+      <c r="W2" s="116"/>
+      <c r="X2" s="116"/>
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
     </row>
     <row r="3" spans="1:64" s="15" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4"/>
@@ -1884,102 +1887,102 @@
       <c r="A4" s="5"/>
       <c r="B4" s="18"/>
       <c r="E4" s="19"/>
-      <c r="I4" s="110">
+      <c r="I4" s="120">
         <f>I5</f>
         <v>45936</v>
       </c>
-      <c r="J4" s="110"/>
-      <c r="K4" s="110"/>
-      <c r="L4" s="110"/>
-      <c r="M4" s="110"/>
-      <c r="N4" s="110"/>
-      <c r="O4" s="111"/>
-      <c r="P4" s="109">
+      <c r="J4" s="120"/>
+      <c r="K4" s="120"/>
+      <c r="L4" s="120"/>
+      <c r="M4" s="120"/>
+      <c r="N4" s="120"/>
+      <c r="O4" s="121"/>
+      <c r="P4" s="119">
         <f>P5</f>
         <v>45943</v>
       </c>
-      <c r="Q4" s="110"/>
-      <c r="R4" s="110"/>
-      <c r="S4" s="110"/>
-      <c r="T4" s="110"/>
-      <c r="U4" s="110"/>
-      <c r="V4" s="111"/>
-      <c r="W4" s="109">
+      <c r="Q4" s="120"/>
+      <c r="R4" s="120"/>
+      <c r="S4" s="120"/>
+      <c r="T4" s="120"/>
+      <c r="U4" s="120"/>
+      <c r="V4" s="121"/>
+      <c r="W4" s="119">
         <f>W5</f>
         <v>45950</v>
       </c>
-      <c r="X4" s="110"/>
-      <c r="Y4" s="110"/>
-      <c r="Z4" s="110"/>
-      <c r="AA4" s="110"/>
-      <c r="AB4" s="110"/>
-      <c r="AC4" s="111"/>
-      <c r="AD4" s="109">
+      <c r="X4" s="120"/>
+      <c r="Y4" s="120"/>
+      <c r="Z4" s="120"/>
+      <c r="AA4" s="120"/>
+      <c r="AB4" s="120"/>
+      <c r="AC4" s="121"/>
+      <c r="AD4" s="119">
         <f>AD5</f>
         <v>45957</v>
       </c>
-      <c r="AE4" s="110"/>
-      <c r="AF4" s="110"/>
-      <c r="AG4" s="110"/>
-      <c r="AH4" s="110"/>
-      <c r="AI4" s="110"/>
-      <c r="AJ4" s="111"/>
-      <c r="AK4" s="109">
+      <c r="AE4" s="120"/>
+      <c r="AF4" s="120"/>
+      <c r="AG4" s="120"/>
+      <c r="AH4" s="120"/>
+      <c r="AI4" s="120"/>
+      <c r="AJ4" s="121"/>
+      <c r="AK4" s="119">
         <f>AK5</f>
         <v>45964</v>
       </c>
-      <c r="AL4" s="110"/>
-      <c r="AM4" s="110"/>
-      <c r="AN4" s="110"/>
-      <c r="AO4" s="110"/>
-      <c r="AP4" s="110"/>
-      <c r="AQ4" s="111"/>
-      <c r="AR4" s="109">
+      <c r="AL4" s="120"/>
+      <c r="AM4" s="120"/>
+      <c r="AN4" s="120"/>
+      <c r="AO4" s="120"/>
+      <c r="AP4" s="120"/>
+      <c r="AQ4" s="121"/>
+      <c r="AR4" s="119">
         <f>AR5</f>
         <v>45971</v>
       </c>
-      <c r="AS4" s="110"/>
-      <c r="AT4" s="110"/>
-      <c r="AU4" s="110"/>
-      <c r="AV4" s="110"/>
-      <c r="AW4" s="110"/>
-      <c r="AX4" s="111"/>
-      <c r="AY4" s="109">
+      <c r="AS4" s="120"/>
+      <c r="AT4" s="120"/>
+      <c r="AU4" s="120"/>
+      <c r="AV4" s="120"/>
+      <c r="AW4" s="120"/>
+      <c r="AX4" s="121"/>
+      <c r="AY4" s="119">
         <f>AY5</f>
         <v>45978</v>
       </c>
-      <c r="AZ4" s="110"/>
-      <c r="BA4" s="110"/>
-      <c r="BB4" s="110"/>
-      <c r="BC4" s="110"/>
-      <c r="BD4" s="110"/>
-      <c r="BE4" s="111"/>
-      <c r="BF4" s="109">
+      <c r="AZ4" s="120"/>
+      <c r="BA4" s="120"/>
+      <c r="BB4" s="120"/>
+      <c r="BC4" s="120"/>
+      <c r="BD4" s="120"/>
+      <c r="BE4" s="121"/>
+      <c r="BF4" s="119">
         <f>BF5</f>
         <v>45985</v>
       </c>
-      <c r="BG4" s="110"/>
-      <c r="BH4" s="110"/>
-      <c r="BI4" s="110"/>
-      <c r="BJ4" s="110"/>
-      <c r="BK4" s="110"/>
-      <c r="BL4" s="110"/>
+      <c r="BG4" s="120"/>
+      <c r="BH4" s="120"/>
+      <c r="BI4" s="120"/>
+      <c r="BJ4" s="120"/>
+      <c r="BK4" s="120"/>
+      <c r="BL4" s="120"/>
     </row>
     <row r="5" spans="1:64" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="121"/>
-      <c r="B5" s="119" t="s">
+      <c r="A5" s="115"/>
+      <c r="B5" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="117" t="s">
+      <c r="C5" s="111" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="112" t="s">
+      <c r="D5" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="112" t="s">
+      <c r="E5" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="112" t="s">
+      <c r="F5" s="109" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="20">
@@ -2208,12 +2211,12 @@
       </c>
     </row>
     <row r="6" spans="1:64" s="15" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="121"/>
-      <c r="B6" s="120"/>
-      <c r="C6" s="118"/>
-      <c r="D6" s="113"/>
-      <c r="E6" s="113"/>
-      <c r="F6" s="113"/>
+      <c r="A6" s="115"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="110"/>
+      <c r="E6" s="110"/>
+      <c r="F6" s="110"/>
       <c r="I6" s="23" t="str">
         <f t="shared" ref="I6:AN6" si="3">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>M</v>
@@ -4311,7 +4314,9 @@
       <c r="C31" s="92" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="93"/>
+      <c r="D31" s="93">
+        <v>1</v>
+      </c>
       <c r="E31" s="94">
         <f>F29</f>
         <v>45982</v>
@@ -4390,7 +4395,9 @@
       <c r="C32" s="92" t="s">
         <v>13</v>
       </c>
-      <c r="D32" s="93"/>
+      <c r="D32" s="93">
+        <v>1</v>
+      </c>
       <c r="E32" s="94">
         <f>E31</f>
         <v>45982</v>
@@ -4540,7 +4547,9 @@
       <c r="C34" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="D34" s="102"/>
+      <c r="D34" s="102" t="s">
+        <v>103</v>
+      </c>
       <c r="E34" s="103">
         <f>F32</f>
         <v>45989</v>
@@ -4619,7 +4628,9 @@
       <c r="C35" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="D35" s="102"/>
+      <c r="D35" s="102" t="s">
+        <v>103</v>
+      </c>
       <c r="E35" s="103">
         <f>E34</f>
         <v>45989</v>
@@ -4698,7 +4709,9 @@
       <c r="C36" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="102"/>
+      <c r="D36" s="102">
+        <v>1</v>
+      </c>
       <c r="E36" s="103">
         <f>E35</f>
         <v>45989</v>
@@ -4777,7 +4790,9 @@
       <c r="C37" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="D37" s="102"/>
+      <c r="D37" s="102">
+        <v>1</v>
+      </c>
       <c r="E37" s="103">
         <f>E36</f>
         <v>45989</v>
@@ -4927,7 +4942,9 @@
       <c r="C39" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="D39" s="65"/>
+      <c r="D39" s="65">
+        <v>1</v>
+      </c>
       <c r="E39" s="66">
         <f>E37</f>
         <v>45989</v>
@@ -5077,7 +5094,9 @@
       <c r="C41" s="104" t="s">
         <v>15</v>
       </c>
-      <c r="D41" s="93"/>
+      <c r="D41" s="93">
+        <v>1</v>
+      </c>
       <c r="E41" s="94">
         <f>F39</f>
         <v>45996</v>
@@ -5150,16 +5169,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="Q2:Z2"/>
-    <mergeCell ref="Q1:Z1"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="I2:O2"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
@@ -5168,6 +5177,16 @@
     <mergeCell ref="AK4:AQ4"/>
     <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="Q2:Z2"/>
+    <mergeCell ref="Q1:Z1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="I2:O2"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A5:A6"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D41">
     <cfRule type="dataBar" priority="26">
@@ -5843,6 +5862,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006B8B2E08FBA2934085025AE2CC2D4FCF" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8d5915535425329bcbd771e38b5089a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d9b4d3a9-89d7-4752-9f66-1c4049782483" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a4a6479488fcfa1ea26509531871ed87" ns3:_="">
     <xsd:import namespace="d9b4d3a9-89d7-4752-9f66-1c4049782483"/>
@@ -5992,15 +6020,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
   <ds:schemaRefs>
@@ -6011,6 +6030,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E186200E-CA11-482F-967A-1FD62478FEA5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6028,14 +6055,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>